<commit_message>
adding resume and reports
</commit_message>
<xml_diff>
--- a/Resources/TestData/Naukri.xlsx
+++ b/Resources/TestData/Naukri.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sushh\Desktop\Divya\Naukri\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B4509C-E5B1-4CF5-A747-F6DC1F157664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B6CFFF-4CD3-46C4-9D58-0D5AB27C42B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
     <t>NewRead2</t>
   </si>
   <si>
-    <t>C:\\Users\\sushh\\Desktop\\Divya\\Naukri\\Resources\\TestData\\Divya.docx</t>
+    <t>C:\\Users\\sushh\\Desktop\\Divya\\Naukri\\Resources\\TestData\\Resume_Divya.pdf</t>
   </si>
 </sst>
 </file>

</xml_diff>